<commit_message>
Updates weight loss plan spreadsheet
Introduces changes to the weight loss tracking spreadsheet to support revised planning, improved progress tracking, or updated calculation logic.
</commit_message>
<xml_diff>
--- a/excel/weight_loss_plan.xlsx
+++ b/excel/weight_loss_plan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
   <si>
     <t>Week</t>
   </si>
@@ -195,7 +195,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -225,6 +225,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1113,9 +1116,11 @@
       </c>
       <c r="F13">
         <f t="shared" si="0"/>
-        <v>81.569999999999993</v>
-      </c>
-      <c r="G13" s="2"/>
+        <v>81.59</v>
+      </c>
+      <c r="G13" s="2">
+        <v>3</v>
+      </c>
       <c r="H13" s="1">
         <v>81.8</v>
       </c>
@@ -1134,27 +1139,51 @@
       <c r="M13" s="17">
         <v>81.400000000000006</v>
       </c>
-      <c r="N13" s="1"/>
+      <c r="N13" s="1">
+        <v>81.7</v>
+      </c>
     </row>
     <row r="14" spans="1:14">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
+      <c r="B14" s="18">
+        <v>2700</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>26</v>
+      </c>
       <c r="E14" s="1">
         <v>82.04</v>
       </c>
-      <c r="F14" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="L14" s="1"/>
+      <c r="F14">
+        <f>ROUND(AVERAGE(I14:N14), 2)</f>
+        <v>80.97</v>
+      </c>
+      <c r="G14" s="2">
+        <v>5</v>
+      </c>
+      <c r="H14" s="18">
+        <v>81.7</v>
+      </c>
+      <c r="I14" s="18">
+        <v>81.7</v>
+      </c>
+      <c r="J14" s="1">
+        <v>81.400000000000006</v>
+      </c>
+      <c r="K14" s="18">
+        <v>81.05</v>
+      </c>
+      <c r="L14" s="1">
+        <v>80.5</v>
+      </c>
+      <c r="M14" s="18">
+        <v>80.2</v>
+      </c>
       <c r="N14" s="1"/>
     </row>
     <row r="15" spans="1:14">
@@ -1262,10 +1291,10 @@
       <c r="B31" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C31" s="18" t="s">
+      <c r="C31" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="D31" s="18"/>
+      <c r="D31" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>